<commit_message>
docs(competitors): refresh completed RFP response for shipped GRC capability
Update 10 compliance descriptions in the completed BPM Tool Functional
Requirements response to reflect the now-shipped Risk & Control (GRC)
feature — Risk-Control Matrix, GRC traceability graph (Risk/Control/
Policy/Regulation/Audit Finding/KRI/KPI), coverage + segregation-of-duties
scans, and control operating-effectiveness proven from mined conformance.

Rows: FR05.02-05 (linkages/traceability), FR02.11 (attributes),
FR06.03/04 (KPI/KRI measures), FR07.27 (lifecycle evidence),
FR11.07/12 (reporting/export). Compliance levels unchanged — only the
descriptions were understating what now ships.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/competitors/BPM Tool Functional Requirements - Diagramatix.xlsx
+++ b/competitors/BPM Tool Functional Requirements - Diagramatix.xlsx
@@ -3759,7 +3759,7 @@
       </c>
       <c r="G9" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Backup/export exposes repository data (objects, roles, attributes, links) and specific structured exports exist (e.g. the Risk-Control Matrix .xlsx).</t>
+          <t xml:space="preserve">The Risk-Control Matrix, Control Register, GRC Register, traceability graph and coverage summary all export to a multi-sheet Excel workbook in the format auditors expect, giving reportable governance output over the repository.</t>
         </is>
       </c>
       <c r="H9" s="39" t="inlineStr">
@@ -3915,7 +3915,7 @@
       </c>
       <c r="G14" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">The model shows roles (lanes) × tasks × associated data objects, and the Risk-Control Matrix demonstrates tabular projection of model data.</t>
+          <t xml:space="preserve">Governance reporting includes a control-coverage summary (risks with no mitigating control), segregation-of-duties findings, and — where mined — per-control operating-effectiveness, all exportable to Excel for audit and compliance review.</t>
         </is>
       </c>
       <c r="H14" s="39" t="inlineStr">
@@ -7714,7 +7714,7 @@
       </c>
       <c r="G13" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Business rules can be recorded as element properties and edited in the Properties panel; the new Risk-Control Matrix provides an aggregated grid for the risk/control subset.</t>
+          <t xml:space="preserve">Risk and control attributes (likelihood, impact, residual score, control type/frequency/owner, framework reference) are held on catalog objects and surfaced against the steps they are attached to, extending the element-attribute model to governance data.</t>
         </is>
       </c>
       <c r="H13" s="39" t="inlineStr">
@@ -8506,7 +8506,7 @@
       </c>
       <c r="G4" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">The Risk &amp; Control feature attaches Risks to process steps, shows them on the model and produces a Risk-Control Matrix.</t>
+          <t xml:space="preserve">Risks are attached to process steps from an org-adopted Risk &amp; Control catalog and shown on the model. The Risk-Control Matrix exports Activity × Risk × Control, a coverage scan flags any risk with no mitigating control, and — where a mined event log exists — control operating-effectiveness is proven from conformance (“bypassed in N of M cases”).</t>
         </is>
       </c>
       <c r="H4" s="39"/>
@@ -8534,7 +8534,7 @@
       </c>
       <c r="G5" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Risk Managers attach and review Risks on process steps via the Risk &amp; Control feature.</t>
+          <t xml:space="preserve">Controls are attached to the steps they govern from the shared catalog, carry type/frequency/owner/framework attributes, and appear on the model. Control-to-risk mitigation is a first-class link, exported in the Risk-Control Matrix and checked by the coverage and segregation-of-duties rules.</t>
         </is>
       </c>
       <c r="H5" s="39"/>
@@ -8562,7 +8562,7 @@
       </c>
       <c r="G6" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Controls carry framework references (e.g. SOX, ISO 27001) and are attached to steps, so regulatory/control activities are marked on the model.</t>
+          <t xml:space="preserve">Regulations and Policies are first-class GRC objects in the catalog, linked to the Risks and Controls that satisfy them via a directed traceability graph (Risk–Control–Policy–Regulation–Audit Finding–KRI–KPI). Controls also carry framework references (e.g. SOX, ISO 27001). Traceability exports to the GRC register.</t>
         </is>
       </c>
       <c r="H6" s="39"/>
@@ -8590,7 +8590,7 @@
       </c>
       <c r="G7" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Control activities are attached to steps via the Risk &amp; Control feature and appear on the model.</t>
+          <t xml:space="preserve">Audit Findings, KRIs and KPIs are catalog objects linked to the Risks, Controls and steps they relate to, giving end-to-end traceability from regulation down to the process activity and its measured performance. The whole graph exports to Excel for auditors.</t>
         </is>
       </c>
       <c r="H7" s="39"/>
@@ -9019,7 +9019,7 @@
       </c>
       <c r="G5" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">KPIs are recorded as attributes on ArchiMate system/application elements or diagram properties.</t>
+          <t xml:space="preserve">KPIs are first-class GRC catalog objects that can be linked to Risks, Controls and process steps, so process performance targets are traceable alongside the risk and control that govern them; they export in the GRC register.</t>
         </is>
       </c>
       <c r="H5" s="39" t="inlineStr">
@@ -9051,7 +9051,7 @@
       </c>
       <c r="G6" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Suggested measures/KPIs attach to model elements as properties, and the Simulator consumes cycle-time/cost measures.</t>
+          <t xml:space="preserve">KRIs (Key Risk Indicators) are first-class catalog objects linked to the Risks they signal and the Controls that mitigate them, so risk indicators are modelled and traceable, not just documented; they export in the GRC register.</t>
         </is>
       </c>
       <c r="H6" s="39"/>
@@ -10066,7 +10066,7 @@
       </c>
       <c r="G29" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Roles are modelled as lanes, responsibility attributes can be added as task properties, and control owners are captured in the Risk &amp; Control feature.</t>
+          <t xml:space="preserve">Where a process has a mined event log, each control’s operating effectiveness is computed from conformance deviations (“bypassed in N of M cases”) and shown against the control — evidence of control performance over the process lifecycle drawn from real execution data.</t>
         </is>
       </c>
       <c r="H29" s="39" t="inlineStr">

</xml_diff>